<commit_message>
New order #1 - MD MONGERUL HAQUE
</commit_message>
<xml_diff>
--- a/orders.xlsx
+++ b/orders.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Orders" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -501,6 +501,46 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-07-29 03:03:08</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MD MONGERUL HAQUE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>01715247588</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>KARIMGANJ MODDHOPARA,KARIMGANJ BAZAR
+PO:KARIMGANJ, KARIMGANJ MUNICIPALITY,KARIMGANJ,KISHOREGANJ</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Pending (COD)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>